<commit_message>
commit 11/10 - 18:22
</commit_message>
<xml_diff>
--- a/censo inep - consolidado.xlsx
+++ b/censo inep - consolidado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathw\Downloads\Dados-Censo-Escolar---INEP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{239BEB9E-7E0C-41C9-81D5-DEE621FF8137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D92501-BA91-420E-83AB-9FA809086353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{41C5916E-F0CC-4781-A461-926F77F1B768}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{41C5916E-F0CC-4781-A461-926F77F1B768}"/>
   </bookViews>
   <sheets>
     <sheet name="matriculas" sheetId="1" r:id="rId1"/>

</xml_diff>